<commit_message>
[UPGRAE] Handover Accesoris / Perintilan
</commit_message>
<xml_diff>
--- a/addons/it_asset/static/excel_templates/handover_template.xlsx
+++ b/addons/it_asset/static/excel_templates/handover_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\10.PROJECT\odoo\addons\it_asset\static\excel_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6D09CE-D6DE-49C7-9E2F-630852CDBD7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08775A1-4362-4D46-AE9A-29D1E288E0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="640" xr2:uid="{893A1DC0-8AB0-4530-A233-231F2C4CEE78}"/>
   </bookViews>
@@ -1306,7 +1306,7 @@
   <dimension ref="A2:AJ47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="37" width="2.7109375" customWidth="1"/>
+    <col min="1" max="36" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:36" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1812,10 +1812,7 @@
       <c r="AJ17" s="2"/>
     </row>
     <row r="18" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="str">
-        <f>" Pada hari ini telah dilakukan serah terima perangkat dengan rincian:"</f>
-        <v xml:space="preserve"> Pada hari ini telah dilakukan serah terima perangkat dengan rincian:</v>
-      </c>
+      <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
       <c r="D18" s="26"/>
@@ -2863,10 +2860,7 @@
     <row r="45" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="19"/>
       <c r="B45" s="19"/>
-      <c r="C45" s="36">
-        <f>I14</f>
-        <v>0</v>
-      </c>
+      <c r="C45" s="36"/>
       <c r="D45" s="36"/>
       <c r="E45" s="36"/>
       <c r="F45" s="36"/>
@@ -2877,10 +2871,7 @@
       <c r="K45" s="36"/>
       <c r="L45" s="36"/>
       <c r="M45" s="19"/>
-      <c r="N45" s="36">
-        <f>Z14</f>
-        <v>0</v>
-      </c>
+      <c r="N45" s="36"/>
       <c r="O45" s="36"/>
       <c r="P45" s="36"/>
       <c r="Q45" s="36"/>
@@ -2909,10 +2900,7 @@
     <row r="46" spans="1:36" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="19"/>
       <c r="B46" s="19"/>
-      <c r="C46" s="37">
-        <f>I15</f>
-        <v>0</v>
-      </c>
+      <c r="C46" s="37"/>
       <c r="D46" s="37"/>
       <c r="E46" s="37"/>
       <c r="F46" s="37"/>
@@ -2923,10 +2911,7 @@
       <c r="K46" s="37"/>
       <c r="L46" s="37"/>
       <c r="M46" s="19"/>
-      <c r="N46" s="37">
-        <f>Z15</f>
-        <v>0</v>
-      </c>
+      <c r="N46" s="37"/>
       <c r="O46" s="37"/>
       <c r="P46" s="37"/>
       <c r="Q46" s="37"/>
@@ -2991,7 +2976,7 @@
       <c r="AJ47" s="19"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="81">
     <mergeCell ref="N5:S5"/>
     <mergeCell ref="W2:AI2"/>

</xml_diff>